<commit_message>
Version with fixed b coefficients in airfoils
</commit_message>
<xml_diff>
--- a/export/Приложение_А.xlsx
+++ b/export/Приложение_А.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH14"/>
+  <dimension ref="A1:BH12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -800,28 +800,28 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.61</v>
+        <v>0.7196</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.3858</v>
+        <v>0.5546</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0.45</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>156.3</v>
+        <v>172.9</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.8575</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.2585</v>
+        <v>0.2511</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>0.99</v>
@@ -830,151 +830,151 @@
         <v>0.5</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>0.5</v>
+        <v>0.65</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>62.747</v>
+        <v>58.773</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>31201.452</v>
+        <v>37067.556</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>30889.437</v>
+        <v>36696.88</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>26488.53</v>
+        <v>31468.57</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>318.7</v>
+        <v>324.4</v>
       </c>
       <c r="R2" s="2" t="n">
         <v>100.713</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>136.799</v>
+        <v>144.49</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>1.3583</v>
+        <v>1.4347</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>310.726</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>1.061</v>
+        <v>1.013</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>0.7906</v>
+        <v>0.8434</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.2318</v>
+        <v>0.2728</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.6506999999999999</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>0.3539</v>
+        <v>0.3351</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.5272</v>
+        <v>0.6036</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>0.2943</v>
+        <v>0.2655</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>0.6087</v>
+        <v>0.732</v>
       </c>
       <c r="AD2" s="2" t="n">
-        <v>0.8278</v>
+        <v>0.8763</v>
       </c>
       <c r="AE2" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AF2" s="2" t="n">
-        <v>0.2436</v>
+        <v>0.2814</v>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>60.754</v>
+        <v>56.99</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>0.436</v>
+        <v>0.434</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>151.5</v>
+        <v>166.8</v>
       </c>
       <c r="AJ2" s="2" t="n">
         <v>6</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>1.327</v>
+        <v>1.325</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>0.8092</v>
+        <v>0.8598</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>0.4327</v>
+        <v>0.4344</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.5459000000000001</v>
+        <v>0.5596</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>38.403</v>
+        <v>37.819</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>38.846</v>
+        <v>38.264</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>58.685</v>
+        <v>55.351</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>19.839</v>
+        <v>17.087</v>
       </c>
       <c r="AS2" s="2" t="n">
-        <v>22.351</v>
+        <v>19.171</v>
       </c>
       <c r="AT2" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>150.3</v>
+        <v>166.9</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>175.864</v>
+        <v>202.195</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>242.025</v>
+        <v>272.192</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>249.258</v>
+        <v>279.196</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>175.977</v>
+        <v>202.883</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>318.7</v>
+        <v>324.4</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>272.6</v>
+        <v>267.7</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>0.881</v>
+        <v>0.9546</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>0.8256</v>
+        <v>0.8963</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>0.7527</v>
+        <v>0.8509</v>
       </c>
       <c r="BE2" s="2" t="n">
-        <v>0.7093</v>
+        <v>0.8004</v>
       </c>
       <c r="BF2" s="2" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.8038</v>
       </c>
       <c r="BG2" s="2" t="n">
-        <v>0.6611</v>
+        <v>0.7658</v>
       </c>
       <c r="BH2" s="2" t="n">
-        <v>0.5558</v>
+        <v>0.6909</v>
       </c>
     </row>
     <row r="3">
@@ -982,181 +982,181 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.6395</v>
+        <v>0.7477</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.472</v>
+        <v>0.6245000000000001</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.436</v>
+        <v>0.434</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>151.5</v>
+        <v>166.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.8658</v>
+        <v>0.8653</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.282</v>
+        <v>0.2747</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.986</v>
+        <v>0.985</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>0.6117</v>
+        <v>0.7318</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>60.734</v>
+        <v>57.045</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>34038.583</v>
+        <v>40557.559</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>33556.369</v>
+        <v>39949.195</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>29054.275</v>
+        <v>34567.937</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>352</v>
+        <v>364.1</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>136.799</v>
+        <v>144.49</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>185.342</v>
+        <v>205.536</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>1.3549</v>
+        <v>1.4225</v>
       </c>
       <c r="U3" s="2" t="n">
-        <v>326.828</v>
+        <v>329.763</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>1.324</v>
+        <v>1.326</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>0.8289</v>
+        <v>0.8762</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.2443</v>
+        <v>0.2814</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>0.5313</v>
+        <v>0.6026</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>0.2926</v>
+        <v>0.2656</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.4915</v>
+        <v>0.5548</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>0.2446</v>
+        <v>0.2126</v>
       </c>
       <c r="AC3" s="2" t="n">
-        <v>0.6905</v>
+        <v>0.7926</v>
       </c>
       <c r="AD3" s="2" t="n">
-        <v>0.8593</v>
+        <v>0.9023</v>
       </c>
       <c r="AE3" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AF3" s="2" t="n">
-        <v>0.2527</v>
+        <v>0.2867</v>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>59.32</v>
+        <v>55.853</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>0.4265</v>
+        <v>0.4231</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>148.2</v>
+        <v>162.6</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>6.333</v>
+        <v>6.4</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>1.653</v>
+        <v>1.722</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>0.8441</v>
+        <v>0.8893</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>0.4178</v>
+        <v>0.4173</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.574</v>
+        <v>0.5862000000000001</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>36.049</v>
+        <v>35.45</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>36.721</v>
+        <v>36.113</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>57.121</v>
+        <v>54.012</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>20.401</v>
+        <v>17.899</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>23.271</v>
+        <v>20.403</v>
       </c>
       <c r="AT3" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>145.2</v>
+        <v>160.4</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>173.657</v>
+        <v>198.727</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>246.666</v>
+        <v>276.474</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>253.368</v>
+        <v>282.931</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>172.845</v>
+        <v>198.176</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>352</v>
+        <v>364.1</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>303.7</v>
+        <v>304.9</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>0.8196</v>
+        <v>0.8845</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>0.7736</v>
+        <v>0.8349</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>0.7251</v>
+        <v>0.8082</v>
       </c>
       <c r="BE3" s="2" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.7639</v>
       </c>
       <c r="BF3" s="2" t="n">
-        <v>0.6793</v>
+        <v>0.7744</v>
       </c>
       <c r="BG3" s="2" t="n">
-        <v>0.6502</v>
+        <v>0.7395</v>
       </c>
       <c r="BH3" s="2" t="n">
-        <v>0.6542</v>
+        <v>0.7634</v>
       </c>
     </row>
     <row r="4">
@@ -1164,181 +1164,181 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.6649</v>
+        <v>0.7708</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.5375</v>
+        <v>0.6783</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.4265</v>
+        <v>0.4231</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>148.2</v>
+        <v>162.6</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.8736</v>
+        <v>0.8726</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.3041</v>
+        <v>0.2967</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.982</v>
+        <v>0.98</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0.6966</v>
+        <v>0.7949000000000001</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>59.18</v>
+        <v>55.812</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>36701.088</v>
+        <v>43805.585</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>36028.235</v>
+        <v>42929.473</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>31475.912</v>
+        <v>37458.473</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>387.6</v>
+        <v>406.5</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>185.342</v>
+        <v>205.536</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>249.724</v>
+        <v>289.039</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>1.3474</v>
+        <v>1.4063</v>
       </c>
       <c r="U4" s="2" t="n">
-        <v>343.406</v>
+        <v>349.224</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>1.645</v>
+        <v>1.715</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>0.8618</v>
+        <v>0.9033</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>0.2545</v>
+        <v>0.2874</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>0.5024999999999999</v>
+        <v>0.5627</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>0.2407</v>
+        <v>0.2105</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.4671</v>
+        <v>0.5208</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>0.203</v>
+        <v>0.171</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>0.7522</v>
+        <v>0.8372000000000001</v>
       </c>
       <c r="AD4" s="2" t="n">
-        <v>0.8848</v>
+        <v>0.9222</v>
       </c>
       <c r="AE4" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AF4" s="2" t="n">
-        <v>0.2686</v>
+        <v>0.2982</v>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>57.25</v>
+        <v>54.181</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.4182</v>
+        <v>0.4135</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>145.3</v>
+        <v>158.9</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>6.667</v>
+        <v>6.8</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>2.043</v>
+        <v>2.203</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>0.8733</v>
+        <v>0.9127</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>0.4073</v>
+        <v>0.4054</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.5993000000000001</v>
+        <v>0.6095</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>34.204</v>
+        <v>33.628</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>35.082</v>
+        <v>34.487</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>56.073</v>
+        <v>53.204</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>20.991</v>
+        <v>18.717</v>
       </c>
       <c r="AS4" s="2" t="n">
-        <v>23.046</v>
+        <v>20.554</v>
       </c>
       <c r="AT4" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>141.5</v>
+        <v>155.8</v>
       </c>
       <c r="AV4" s="2" t="n">
-        <v>172.554</v>
+        <v>196.519</v>
       </c>
       <c r="AW4" s="2" t="n">
-        <v>251.749</v>
+        <v>281.26</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>257.829</v>
+        <v>287.098</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>170.556</v>
+        <v>194.512</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>387.6</v>
+        <v>406.5</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>337.2</v>
+        <v>345</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>0.7705</v>
+        <v>0.8262</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>0.7314000000000001</v>
+        <v>0.7841</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>0.7006</v>
+        <v>0.7715</v>
       </c>
       <c r="BE4" s="2" t="n">
-        <v>0.6659</v>
+        <v>0.7329</v>
       </c>
       <c r="BF4" s="2" t="n">
-        <v>0.6651</v>
+        <v>0.746</v>
       </c>
       <c r="BG4" s="2" t="n">
-        <v>0.6377</v>
+        <v>0.714</v>
       </c>
       <c r="BH4" s="2" t="n">
-        <v>0.7274</v>
+        <v>0.8174</v>
       </c>
     </row>
     <row r="5">
@@ -1346,181 +1346,181 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.6847</v>
+        <v>0.7879</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.585</v>
+        <v>0.7166</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.4182</v>
+        <v>0.4135</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>145.3</v>
+        <v>158.9</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.8709</v>
+        <v>0.8692</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.3075</v>
+        <v>0.3005</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0.978</v>
+        <v>0.975</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0.7582</v>
+        <v>0.8399</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>57.109</v>
+        <v>54.13</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>37113.861</v>
+        <v>44357.527</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>36278.799</v>
+        <v>43248.589</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>31595.503</v>
+        <v>37592.953</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>423.4</v>
+        <v>449</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>249.724</v>
+        <v>289.039</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>328.044</v>
+        <v>393.286</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>1.3136</v>
+        <v>1.3607</v>
       </c>
       <c r="U5" s="2" t="n">
-        <v>360.268</v>
+        <v>368.861</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>2.032</v>
+        <v>2.192</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>0.8874</v>
+        <v>0.9234</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>0.2704</v>
+        <v>0.299</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>0.4803</v>
+        <v>0.5316</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>0.1988</v>
+        <v>0.1685</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.4449</v>
+        <v>0.4909</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>0.1713</v>
+        <v>0.1407</v>
       </c>
       <c r="AC5" s="2" t="n">
-        <v>0.796</v>
+        <v>0.8683</v>
       </c>
       <c r="AD5" s="2" t="n">
-        <v>0.9038</v>
+        <v>0.9364</v>
       </c>
       <c r="AE5" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AF5" s="2" t="n">
-        <v>0.2801</v>
+        <v>0.306</v>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>55.674</v>
+        <v>52.892</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>0.4105</v>
+        <v>0.4047</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>142.6</v>
+        <v>155.5</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>2.478</v>
+        <v>2.75</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>0.8956</v>
+        <v>0.9298999999999999</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>0.398</v>
+        <v>0.3948</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.6113</v>
+        <v>0.62</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>33.07</v>
+        <v>32.486</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>34.131</v>
+        <v>33.515</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>54.463</v>
+        <v>51.867</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>20.333</v>
+        <v>18.352</v>
       </c>
       <c r="AS5" s="2" t="n">
-        <v>22.604</v>
+        <v>20.406</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>138.3</v>
+        <v>151.7</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>173.021</v>
+        <v>196.07</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>253.431</v>
+        <v>282.419</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>258.94</v>
+        <v>287.751</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>169.939</v>
+        <v>192.839</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>423.4</v>
+        <v>449</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>372.9</v>
+        <v>387.6</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>0.7216</v>
+        <v>0.7696</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.7348</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>0.6696</v>
+        <v>0.7302</v>
       </c>
       <c r="BE5" s="2" t="n">
-        <v>0.6399</v>
+        <v>0.6977</v>
       </c>
       <c r="BF5" s="2" t="n">
-        <v>0.6413</v>
+        <v>0.7103</v>
       </c>
       <c r="BG5" s="2" t="n">
-        <v>0.6165</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="BH5" s="2" t="n">
-        <v>0.78</v>
+        <v>0.8554</v>
       </c>
     </row>
     <row r="6">
@@ -1528,181 +1528,181 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.6993</v>
+        <v>0.8001</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.6186</v>
+        <v>0.7432</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.4105</v>
+        <v>0.4047</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>142.6</v>
+        <v>155.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.8681</v>
+        <v>0.8658</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0.3105</v>
+        <v>0.3038</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.973</v>
+        <v>0.97</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0.8018</v>
+        <v>0.871</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>55.526</v>
+        <v>52.828</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>37479.232</v>
+        <v>44843.01</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>36479.786</v>
+        <v>43497.72</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>31667.854</v>
+        <v>37659.32</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>459.2</v>
+        <v>491.5</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>328.044</v>
+        <v>393.286</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>421.697</v>
+        <v>520.6130000000001</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>1.2855</v>
+        <v>1.3238</v>
       </c>
       <c r="U6" s="2" t="n">
-        <v>376.37</v>
+        <v>387.471</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>2.464</v>
+        <v>2.734</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>0.9063</v>
+        <v>0.9377</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.2819</v>
+        <v>0.3069</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>0.4597</v>
+        <v>0.5037</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>0.167</v>
+        <v>0.138</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.4247</v>
+        <v>0.4643</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>0.1466</v>
+        <v>0.1181</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>0.8285</v>
+        <v>0.8908</v>
       </c>
       <c r="AD6" s="2" t="n">
-        <v>0.9183</v>
+        <v>0.947</v>
       </c>
       <c r="AE6" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AF6" s="2" t="n">
-        <v>0.2886</v>
+        <v>0.3115</v>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>54.405</v>
+        <v>51.833</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>0.4033</v>
+        <v>0.3965</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>140.1</v>
+        <v>152.3</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>7.333</v>
+        <v>7.6</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>2.96</v>
+        <v>3.361</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>0.9123</v>
+        <v>0.9423</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>0.3894</v>
+        <v>0.385</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.6204</v>
+        <v>0.6277</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>32.116</v>
+        <v>31.519</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>33.321</v>
+        <v>32.684</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>53.142</v>
+        <v>50.741</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>19.822</v>
+        <v>18.057</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>22.289</v>
+        <v>20.314</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>135.3</v>
+        <v>147.9</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>173.008</v>
+        <v>195.16</v>
       </c>
       <c r="AW6" s="2" t="n">
-        <v>254.478</v>
+        <v>282.929</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>259.636</v>
+        <v>287.977</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>169.087</v>
+        <v>191.024</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>459.2</v>
+        <v>491.5</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>408.7</v>
+        <v>430.4</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.7239</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>0.6539</v>
+        <v>0.6941000000000001</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>0.6419</v>
+        <v>0.6944</v>
       </c>
       <c r="BE6" s="2" t="n">
-        <v>0.6158</v>
+        <v>0.6662</v>
       </c>
       <c r="BF6" s="2" t="n">
-        <v>0.6188</v>
+        <v>0.6784</v>
       </c>
       <c r="BG6" s="2" t="n">
-        <v>0.5961</v>
+        <v>0.6531</v>
       </c>
       <c r="BH6" s="2" t="n">
-        <v>0.8179</v>
+        <v>0.8823</v>
       </c>
     </row>
     <row r="7">
@@ -1710,181 +1710,181 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.7104</v>
+        <v>0.8091</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.6435</v>
+        <v>0.7624</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.4033</v>
+        <v>0.3965</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>140.1</v>
+        <v>152.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0.8652</v>
+        <v>0.8622</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.3132</v>
+        <v>0.3067</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0.969</v>
+        <v>0.965</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>0.834</v>
+        <v>0.8935</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>54.258</v>
+        <v>51.764</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>37810.268</v>
+        <v>45280.09</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>36644.452</v>
+        <v>43695.286</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>31704.361</v>
+        <v>37673.688</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>494.9</v>
+        <v>533.9</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>421.697</v>
+        <v>520.6130000000001</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>532.074</v>
+        <v>673.3339999999999</v>
       </c>
       <c r="T7" s="2" t="n">
-        <v>1.2617</v>
+        <v>1.2933</v>
       </c>
       <c r="U7" s="2" t="n">
-        <v>391.769</v>
+        <v>405.144</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>2.942</v>
+        <v>3.342</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>0.9208</v>
+        <v>0.9483</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.2903</v>
+        <v>0.3124</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.4407</v>
+        <v>0.4787</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>0.1423</v>
+        <v>0.1153</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>0.4061</v>
+        <v>0.4406</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>0.1271</v>
+        <v>0.1007</v>
       </c>
       <c r="AC7" s="2" t="n">
-        <v>0.8534</v>
+        <v>0.9077</v>
       </c>
       <c r="AD7" s="2" t="n">
-        <v>0.9296</v>
+        <v>0.955</v>
       </c>
       <c r="AE7" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AF7" s="2" t="n">
-        <v>0.2949</v>
+        <v>0.3155</v>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>53.347</v>
+        <v>50.927</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>0.3965</v>
+        <v>0.3886</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>137.7</v>
+        <v>149.3</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>7.667</v>
+        <v>8</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>3.487</v>
+        <v>4.039</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>0.9252</v>
+        <v>0.9516</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>0.3813</v>
+        <v>0.3757</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>0.6274999999999999</v>
+        <v>0.6336000000000001</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>31.283</v>
+        <v>30.663</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>32.608</v>
+        <v>31.945</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>52.017</v>
+        <v>49.752</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>19.409</v>
+        <v>17.806</v>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>22.064</v>
+        <v>20.263</v>
       </c>
       <c r="AT7" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>132.5</v>
+        <v>144.3</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>172.642</v>
+        <v>193.947</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>255.087</v>
+        <v>283.023</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>260.03</v>
+        <v>287.916</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>168.054</v>
+        <v>189.111</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>494.9</v>
+        <v>533.9</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>444.6</v>
+        <v>473.3</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>0.6489</v>
+        <v>0.6859</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>0.624</v>
+        <v>0.6597</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>0.6171</v>
+        <v>0.663</v>
       </c>
       <c r="BE7" s="2" t="n">
-        <v>0.5937</v>
+        <v>0.6381</v>
       </c>
       <c r="BF7" s="2" t="n">
-        <v>0.5979</v>
+        <v>0.6499</v>
       </c>
       <c r="BG7" s="2" t="n">
-        <v>0.5769</v>
+        <v>0.627</v>
       </c>
       <c r="BH7" s="2" t="n">
-        <v>0.8463000000000001</v>
+        <v>0.902</v>
       </c>
     </row>
     <row r="8">
@@ -1892,181 +1892,181 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.7191</v>
+        <v>0.8159</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.6624</v>
+        <v>0.7768</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>347.43</v>
+        <v>384.23</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.3965</v>
+        <v>0.3886</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>137.7</v>
+        <v>149.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.8622</v>
+        <v>0.8585</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.3158</v>
+        <v>0.3094</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.965</v>
+        <v>0.96</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0.8586</v>
+        <v>0.9104</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>53.203</v>
+        <v>50.856</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>38114.316</v>
+        <v>45678.947</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>36780.315</v>
+        <v>43851.789</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>31711.661</v>
+        <v>37645.531</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>530.6</v>
+        <v>576.1</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>532.074</v>
+        <v>673.3339999999999</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>660.552</v>
+        <v>853.73</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>1.2415</v>
+        <v>1.2679</v>
       </c>
       <c r="U8" s="2" t="n">
-        <v>406.517</v>
+        <v>421.963</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>3.466</v>
+        <v>4.015</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.9562</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.2966</v>
+        <v>0.3163</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>0.4232</v>
+        <v>0.4563</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>0.1229</v>
+        <v>0.0979</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>0.3891</v>
+        <v>0.4192</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>0.1114</v>
+        <v>0.0871</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>0.8728</v>
+        <v>0.9191</v>
       </c>
       <c r="AD8" s="2" t="n">
-        <v>0.9386</v>
+        <v>0.9604</v>
       </c>
       <c r="AE8" s="2" t="n">
-        <v>347.43</v>
+        <v>379.86</v>
       </c>
       <c r="AF8" s="2" t="n">
-        <v>0.2998</v>
+        <v>0.3178</v>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>52.438</v>
+        <v>50.125</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>0.3899</v>
+        <v>0.3811</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>135.5</v>
+        <v>144.8</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>4.062</v>
+        <v>4.784</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>0.9353</v>
+        <v>0.9583</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>0.3735</v>
+        <v>0.3668</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>0.6332</v>
+        <v>0.6385</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>30.534</v>
+        <v>29.874</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>31.964</v>
+        <v>31.272</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>51.029</v>
+        <v>48.913</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>19.065</v>
+        <v>17.641</v>
       </c>
       <c r="AS8" s="2" t="n">
-        <v>21.904</v>
+        <v>20.251</v>
       </c>
       <c r="AT8" s="2" t="n">
-        <v>347.43</v>
+        <v>382.04</v>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>129.7</v>
+        <v>140.9</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>172.023</v>
+        <v>192.539</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>255.389</v>
+        <v>282.93</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>260.204</v>
+        <v>287.664</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>166.888</v>
+        <v>186.976</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>530.6</v>
+        <v>576.1</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>480.6</v>
+        <v>516.1</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>0.6205000000000001</v>
+        <v>0.6466</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>0.5981</v>
+        <v>0.6253</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>0.5947</v>
+        <v>0.6354</v>
       </c>
       <c r="BE8" s="2" t="n">
-        <v>0.5735</v>
+        <v>0.6131</v>
       </c>
       <c r="BF8" s="2" t="n">
-        <v>0.5785</v>
+        <v>0.6173</v>
       </c>
       <c r="BG8" s="2" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.5982</v>
       </c>
       <c r="BH8" s="2" t="n">
-        <v>0.8682</v>
+        <v>0.9156</v>
       </c>
     </row>
     <row r="9">
@@ -2074,181 +2074,181 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8436</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.7259</v>
+        <v>0.8109</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.6773</v>
+        <v>0.7768</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>347.43</v>
+        <v>379.86</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.3899</v>
+        <v>0.3811</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>135.5</v>
+        <v>144.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.8591</v>
+        <v>0.8546</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.3181</v>
+        <v>0.3119</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.961</v>
+        <v>0.955</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>0.8778</v>
+        <v>0.9209000000000001</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>52.298</v>
+        <v>50.126</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>38396.071</v>
+        <v>46046.107</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>36892.225</v>
+        <v>43974.032</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>31694.147</v>
+        <v>37581.17</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>566.1</v>
+        <v>618</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>660.552</v>
+        <v>853.73</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>808.492</v>
+        <v>1064.033</v>
       </c>
       <c r="T9" s="2" t="n">
-        <v>1.224</v>
+        <v>1.2463</v>
       </c>
       <c r="U9" s="2" t="n">
-        <v>420.663</v>
+        <v>438.003</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>4.037</v>
+        <v>4.764</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>0.9409</v>
+        <v>0.9612000000000001</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>0.3014</v>
+        <v>0.3184</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>0.407</v>
+        <v>0.4307</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>0.1073</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>0.3734</v>
+        <v>0.3945</v>
       </c>
       <c r="AB9" s="2" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.077</v>
       </c>
       <c r="AC9" s="2" t="n">
-        <v>0.8883</v>
+        <v>0.9275</v>
       </c>
       <c r="AD9" s="2" t="n">
-        <v>0.9458</v>
+        <v>0.9644</v>
       </c>
       <c r="AE9" s="2" t="n">
-        <v>347.43</v>
+        <v>376.33</v>
       </c>
       <c r="AF9" s="2" t="n">
-        <v>0.3036</v>
+        <v>0.3193</v>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>51.637</v>
+        <v>49.498</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>0.3836</v>
+        <v>0.3739</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>133.3</v>
+        <v>140.7</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>8.333</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>4.683</v>
+        <v>5.606</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>0.9433</v>
+        <v>0.9628</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>0.3659</v>
+        <v>0.358</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>0.6378</v>
+        <v>0.6418</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>29.845</v>
+        <v>29.15</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>31.373</v>
+        <v>30.662</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>50.14</v>
+        <v>48.113</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>18.767</v>
+        <v>17.451</v>
       </c>
       <c r="AS9" s="2" t="n">
-        <v>21.792</v>
+        <v>20.348</v>
       </c>
       <c r="AT9" s="2" t="n">
-        <v>347.43</v>
+        <v>378.1</v>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>127.1</v>
+        <v>136</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>171.222</v>
+        <v>188.642</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>255.473</v>
+        <v>279.148</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>260.217</v>
+        <v>283.886</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>165.627</v>
+        <v>182.647</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>566.1</v>
+        <v>618</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>516.5</v>
+        <v>559.1</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>0.5958</v>
+        <v>0.6156</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>0.5753</v>
+        <v>0.5961</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>0.5745</v>
+        <v>0.6034</v>
       </c>
       <c r="BE9" s="2" t="n">
-        <v>0.555</v>
+        <v>0.583</v>
       </c>
       <c r="BF9" s="2" t="n">
-        <v>0.5606</v>
+        <v>0.591</v>
       </c>
       <c r="BG9" s="2" t="n">
-        <v>0.5423</v>
+        <v>0.5732</v>
       </c>
       <c r="BH9" s="2" t="n">
-        <v>0.8854</v>
+        <v>0.9251</v>
       </c>
     </row>
     <row r="10">
@@ -2256,181 +2256,181 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8357</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.7315</v>
+        <v>0.8068</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.6891</v>
+        <v>0.7768</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>347.43</v>
+        <v>376.33</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.3836</v>
+        <v>0.3739</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>133.3</v>
+        <v>140.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.8559</v>
+        <v>0.8506</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.3203</v>
+        <v>0.3142</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.957</v>
+        <v>0.95</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0.8931</v>
+        <v>0.9295</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>51.501</v>
+        <v>49.443</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>38658.792</v>
+        <v>46386.108</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>36983.578</v>
+        <v>44066.802</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>31654.969</v>
+        <v>37485.176</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>601.4</v>
+        <v>659.6</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>808.492</v>
+        <v>1064.033</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>977.231</v>
+        <v>1306.42</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>1.2087</v>
+        <v>1.2278</v>
       </c>
       <c r="U10" s="2" t="n">
-        <v>434.254</v>
+        <v>453.334</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>4.655</v>
+        <v>5.579</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0.9481000000000001</v>
+        <v>0.9654</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>0.3051</v>
+        <v>0.32</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>0.3921</v>
+        <v>0.4085</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>0.0946</v>
+        <v>0.0746</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>0.3589</v>
+        <v>0.3675</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.06859999999999999</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>0.901</v>
+        <v>0.9346</v>
       </c>
       <c r="AD10" s="2" t="n">
-        <v>0.9518</v>
+        <v>0.9679</v>
       </c>
       <c r="AE10" s="2" t="n">
-        <v>347.43</v>
+        <v>373.38</v>
       </c>
       <c r="AF10" s="2" t="n">
-        <v>0.3066</v>
+        <v>0.3093</v>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>50.915</v>
+        <v>49.863</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>0.3775</v>
+        <v>0.3668</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>131.1</v>
+        <v>137</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>8.667</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>5.352</v>
+        <v>6.505</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>0.9499</v>
+        <v>0.9666</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>0.3587</v>
+        <v>0.3494</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>0.6417</v>
+        <v>0.6446</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>29.202</v>
+        <v>28.461</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>30.822</v>
+        <v>30.082</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>49.324</v>
+        <v>47.337</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>18.502</v>
+        <v>17.255</v>
       </c>
       <c r="AS10" s="2" t="n">
-        <v>21.713</v>
+        <v>21.402</v>
       </c>
       <c r="AT10" s="2" t="n">
-        <v>347.43</v>
+        <v>374.86</v>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>124.6</v>
+        <v>131.5</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>170.291</v>
+        <v>185.188</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>255.398</v>
+        <v>275.933</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>260.111</v>
+        <v>280.704</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>164.299</v>
+        <v>178.825</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>601.4</v>
+        <v>659.6</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>552.2</v>
+        <v>601.8</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.574</v>
+        <v>0.5889</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>0.555</v>
+        <v>0.5709</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.5561</v>
+        <v>0.5760999999999999</v>
       </c>
       <c r="BE10" s="2" t="n">
-        <v>0.538</v>
+        <v>0.5571</v>
       </c>
       <c r="BF10" s="2" t="n">
-        <v>0.5442</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="BG10" s="2" t="n">
-        <v>0.5269</v>
+        <v>0.5512</v>
       </c>
       <c r="BH10" s="2" t="n">
-        <v>0.8993</v>
+        <v>0.9331</v>
       </c>
     </row>
     <row r="11">
@@ -2438,181 +2438,181 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8292</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.736</v>
+        <v>0.8034</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.6987</v>
+        <v>0.7768</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>347.43</v>
+        <v>373.38</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.3775</v>
+        <v>0.3668</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>131.1</v>
+        <v>137</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.8526</v>
+        <v>0.8364</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.3223</v>
+        <v>0.3005</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.952</v>
+        <v>0.945</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0.9056</v>
+        <v>0.9368</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>50.783</v>
+        <v>49.8</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>38904.868</v>
+        <v>44367.168</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>37056.887</v>
+        <v>41926.974</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>31596.511</v>
+        <v>35067.072</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>636.5</v>
+        <v>698.9</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>977.231</v>
+        <v>1306.42</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>1168.084</v>
+        <v>1564.88</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>1.1953</v>
+        <v>1.1978</v>
       </c>
       <c r="U11" s="2" t="n">
-        <v>447.332</v>
+        <v>468.019</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>5.319</v>
+        <v>6.472</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.954</v>
+        <v>0.9689</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.308</v>
+        <v>0.31</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.3784</v>
+        <v>0.3832</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>0.3454</v>
+        <v>0.3393</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.0621</v>
       </c>
       <c r="AC11" s="2" t="n">
-        <v>0.9114</v>
+        <v>0.9403</v>
       </c>
       <c r="AD11" s="2" t="n">
-        <v>0.9567</v>
+        <v>0.9706</v>
       </c>
       <c r="AE11" s="2" t="n">
-        <v>347.43</v>
+        <v>371.07</v>
       </c>
       <c r="AF11" s="2" t="n">
-        <v>0.3089</v>
+        <v>0.2892</v>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>50.254</v>
+        <v>51.23</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>0.3715</v>
+        <v>0.36</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>129.1</v>
+        <v>133.6</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>9</v>
+        <v>9.6</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>6.069</v>
+        <v>7.417</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.9553</v>
+        <v>0.9698</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>0.3516</v>
+        <v>0.3411</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>0.645</v>
+        <v>0.6196</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>28.594</v>
+        <v>28.834</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>30.302</v>
+        <v>29.106</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>48.562</v>
+        <v>44.255</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>18.26</v>
+        <v>15.149</v>
       </c>
       <c r="AS11" s="2" t="n">
-        <v>21.66</v>
+        <v>22.396</v>
       </c>
       <c r="AT11" s="2" t="n">
-        <v>347.43</v>
+        <v>372.23</v>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>122.1</v>
+        <v>127.4</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>169.268</v>
+        <v>179.329</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>255.209</v>
+        <v>264.105</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>259.916</v>
+        <v>281.589</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>162.926</v>
+        <v>182.519</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>636.5</v>
+        <v>698.9</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>587.8</v>
+        <v>644.6</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>0.5546</v>
+        <v>0.5707</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>0.5369</v>
+        <v>0.5302</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>0.5394</v>
+        <v>0.5594</v>
       </c>
       <c r="BE11" s="2" t="n">
-        <v>0.5224</v>
+        <v>0.5167</v>
       </c>
       <c r="BF11" s="2" t="n">
-        <v>0.5289</v>
+        <v>0.5567</v>
       </c>
       <c r="BG11" s="2" t="n">
-        <v>0.5125999999999999</v>
+        <v>0.5141</v>
       </c>
       <c r="BH11" s="2" t="n">
-        <v>0.9107</v>
+        <v>0.9397</v>
       </c>
     </row>
     <row r="12">
@@ -2620,545 +2620,181 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.7716</v>
+        <v>0.8241000000000001</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.7398</v>
+        <v>0.8008</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.7066</v>
+        <v>0.7768</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>347.43</v>
+        <v>371.07</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.3715</v>
+        <v>0.36</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>129.1</v>
+        <v>133.6</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.8493000000000001</v>
+        <v>0.8213</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.3242</v>
+        <v>0.2865</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.948</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>0.9157999999999999</v>
+        <v>0.9427</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>50.125</v>
+        <v>51.159</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>39136.126</v>
+        <v>42297.467</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>37114.092</v>
+        <v>39759.619</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>31520.657</v>
+        <v>32653.126</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>671.5</v>
+        <v>735.8</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>1168.084</v>
+        <v>1564.88</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>1382.331</v>
+        <v>1834.831</v>
       </c>
       <c r="T12" s="2" t="n">
-        <v>1.1834</v>
+        <v>1.1725</v>
       </c>
       <c r="U12" s="2" t="n">
-        <v>459.935</v>
+        <v>481.419</v>
       </c>
       <c r="V12" s="2" t="n">
-        <v>6.031</v>
+        <v>7.38</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.9588</v>
+        <v>0.9718</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>0.3103</v>
+        <v>0.2899</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>0.3657</v>
+        <v>0.3563</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0594</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>0.3281</v>
+        <v>0.2503</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>0.0717</v>
+        <v>0.0562</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>0.9195</v>
+        <v>0.9455</v>
       </c>
       <c r="AD12" s="2" t="n">
-        <v>0.9606</v>
+        <v>0.9731</v>
       </c>
       <c r="AE12" s="2" t="n">
-        <v>344.73</v>
+        <v>369.96</v>
       </c>
       <c r="AF12" s="2" t="n">
-        <v>0.2999</v>
+        <v>0.2899</v>
       </c>
       <c r="AG12" s="2" t="n">
-        <v>50.63</v>
+        <v>90</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>0.3657</v>
+        <v>0.3331</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>126.1</v>
+        <v>123.6</v>
       </c>
       <c r="AJ12" s="2" t="n">
-        <v>9.333</v>
+        <v>10</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>6.842</v>
+        <v>8.448</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>0.9597</v>
+        <v>0.9724</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>0.3446</v>
+        <v>0.3331</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>0.6479</v>
+        <v>0.5843</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>28.01</v>
+        <v>29.683</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>29.807</v>
+        <v>27.832</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>47.862</v>
+        <v>40.632</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>18.055</v>
+        <v>12.8</v>
       </c>
       <c r="AS12" s="2" t="n">
-        <v>22.62</v>
+        <v>60.317</v>
       </c>
       <c r="AT12" s="2" t="n">
-        <v>346.08</v>
+        <v>370.51</v>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>119.7</v>
+        <v>123.6</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>168.18</v>
+        <v>171.507</v>
       </c>
       <c r="AW12" s="2" t="n">
-        <v>254.962</v>
+        <v>249.563</v>
       </c>
       <c r="AX12" s="2" t="n">
-        <v>259.655</v>
+        <v>286.125</v>
       </c>
       <c r="AY12" s="2" t="n">
-        <v>161.472</v>
+        <v>189.782</v>
       </c>
       <c r="AZ12" s="2" t="n">
-        <v>671.5</v>
+        <v>735.8</v>
       </c>
       <c r="BA12" s="2" t="n">
-        <v>623.2</v>
+        <v>685.2</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>0.5334</v>
+        <v>0.5618</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>0.5178</v>
+        <v>0.4881</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>0.524</v>
+        <v>0.5521</v>
       </c>
       <c r="BE12" s="2" t="n">
-        <v>0.5081</v>
+        <v>0.4748</v>
       </c>
       <c r="BF12" s="2" t="n">
-        <v>0.5109</v>
+        <v>0.5545</v>
       </c>
       <c r="BG12" s="2" t="n">
-        <v>0.4964</v>
+        <v>0.4747</v>
       </c>
       <c r="BH12" s="2" t="n">
-        <v>0.9194</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>0.7655999999999999</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>0.7367</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>0.7066</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>344.73</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>0.3657</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>126.1</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>0.8357</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>0.3097</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>50.547</v>
-      </c>
-      <c r="N13" s="2" t="n">
-        <v>37386.305</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>35298.903</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>29499.206</v>
-      </c>
-      <c r="Q13" s="2" t="n">
-        <v>704.4</v>
-      </c>
-      <c r="R13" s="2" t="n">
-        <v>1382.331</v>
-      </c>
-      <c r="S13" s="2" t="n">
-        <v>1605.739</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>1.1616</v>
-      </c>
-      <c r="U13" s="2" t="n">
-        <v>472.1</v>
-      </c>
-      <c r="V13" s="2" t="n">
-        <v>6.807</v>
-      </c>
-      <c r="W13" s="2" t="n">
-        <v>0.9623</v>
-      </c>
-      <c r="X13" s="2" t="n">
-        <v>0.3009</v>
-      </c>
-      <c r="Y13" s="2" t="n">
-        <v>0.3458</v>
-      </c>
-      <c r="Z13" s="2" t="n">
-        <v>0.0682</v>
-      </c>
-      <c r="AA13" s="2" t="n">
-        <v>0.3052</v>
-      </c>
-      <c r="AB13" s="2" t="n">
-        <v>0.06619999999999999</v>
-      </c>
-      <c r="AC13" s="2" t="n">
-        <v>0.925</v>
-      </c>
-      <c r="AD13" s="2" t="n">
-        <v>0.9631999999999999</v>
-      </c>
-      <c r="AE13" s="2" t="n">
-        <v>342.61</v>
-      </c>
-      <c r="AF13" s="2" t="n">
-        <v>0.2803</v>
-      </c>
-      <c r="AG13" s="2" t="n">
-        <v>52.094</v>
-      </c>
-      <c r="AH13" s="2" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="AI13" s="2" t="n">
-        <v>123.3</v>
-      </c>
-      <c r="AJ13" s="2" t="n">
-        <v>9.667</v>
-      </c>
-      <c r="AK13" s="2" t="n">
-        <v>7.623</v>
-      </c>
-      <c r="AL13" s="2" t="n">
-        <v>0.9628</v>
-      </c>
-      <c r="AM13" s="2" t="n">
-        <v>0.3376</v>
-      </c>
-      <c r="AN13" s="2" t="n">
-        <v>0.6225000000000001</v>
-      </c>
-      <c r="AO13" s="2" t="n">
-        <v>28.475</v>
-      </c>
-      <c r="AP13" s="2" t="n">
-        <v>28.941</v>
-      </c>
-      <c r="AQ13" s="2" t="n">
-        <v>44.781</v>
-      </c>
-      <c r="AR13" s="2" t="n">
-        <v>15.84</v>
-      </c>
-      <c r="AS13" s="2" t="n">
-        <v>23.619</v>
-      </c>
-      <c r="AT13" s="2" t="n">
-        <v>343.67</v>
-      </c>
-      <c r="AU13" s="2" t="n">
-        <v>116.4</v>
-      </c>
-      <c r="AV13" s="2" t="n">
-        <v>163.264</v>
-      </c>
-      <c r="AW13" s="2" t="n">
-        <v>244.134</v>
-      </c>
-      <c r="AX13" s="2" t="n">
-        <v>260.51</v>
-      </c>
-      <c r="AY13" s="2" t="n">
-        <v>165.243</v>
-      </c>
-      <c r="AZ13" s="2" t="n">
-        <v>704.4</v>
-      </c>
-      <c r="BA13" s="2" t="n">
-        <v>659</v>
-      </c>
-      <c r="BB13" s="2" t="n">
-        <v>0.5199</v>
-      </c>
-      <c r="BC13" s="2" t="n">
-        <v>0.4839</v>
-      </c>
-      <c r="BD13" s="2" t="n">
-        <v>0.512</v>
-      </c>
-      <c r="BE13" s="2" t="n">
-        <v>0.4741</v>
-      </c>
-      <c r="BF13" s="2" t="n">
-        <v>0.5044999999999999</v>
-      </c>
-      <c r="BG13" s="2" t="n">
-        <v>0.4658</v>
-      </c>
-      <c r="BH13" s="2" t="n">
-        <v>0.9258</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>0.7609</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>0.7342</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>0.7066</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>342.61</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>123.3</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>0.8213</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>0.295</v>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="K14" s="2" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>0.9287</v>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>51.984</v>
-      </c>
-      <c r="N14" s="2" t="n">
-        <v>35603.706</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>33467.484</v>
-      </c>
-      <c r="P14" s="2" t="n">
-        <v>27485.625</v>
-      </c>
-      <c r="Q14" s="2" t="n">
-        <v>735.4</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>1605.739</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>1834.832</v>
-      </c>
-      <c r="T14" s="2" t="n">
-        <v>1.1427</v>
-      </c>
-      <c r="U14" s="2" t="n">
-        <v>483.276</v>
-      </c>
-      <c r="V14" s="2" t="n">
-        <v>7.584</v>
-      </c>
-      <c r="W14" s="2" t="n">
-        <v>0.965</v>
-      </c>
-      <c r="X14" s="2" t="n">
-        <v>0.2814</v>
-      </c>
-      <c r="Y14" s="2" t="n">
-        <v>0.3239</v>
-      </c>
-      <c r="Z14" s="2" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="AA14" s="2" t="n">
-        <v>0.2296</v>
-      </c>
-      <c r="AB14" s="2" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="AC14" s="2" t="n">
-        <v>0.9302</v>
-      </c>
-      <c r="AD14" s="2" t="n">
-        <v>0.9658</v>
-      </c>
-      <c r="AE14" s="2" t="n">
-        <v>342.04</v>
-      </c>
-      <c r="AF14" s="2" t="n">
-        <v>0.2814</v>
-      </c>
-      <c r="AG14" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="AH14" s="2" t="n">
-        <v>0.3308</v>
-      </c>
-      <c r="AI14" s="2" t="n">
-        <v>113.3</v>
-      </c>
-      <c r="AJ14" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="AK14" s="2" t="n">
-        <v>8.488</v>
-      </c>
-      <c r="AL14" s="2" t="n">
-        <v>0.9654</v>
-      </c>
-      <c r="AM14" s="2" t="n">
-        <v>0.3308</v>
-      </c>
-      <c r="AN14" s="2" t="n">
-        <v>0.5869</v>
-      </c>
-      <c r="AO14" s="2" t="n">
-        <v>29.41</v>
-      </c>
-      <c r="AP14" s="2" t="n">
-        <v>27.773</v>
-      </c>
-      <c r="AQ14" s="2" t="n">
-        <v>41.152</v>
-      </c>
-      <c r="AR14" s="2" t="n">
-        <v>13.379</v>
-      </c>
-      <c r="AS14" s="2" t="n">
-        <v>60.59</v>
-      </c>
-      <c r="AT14" s="2" t="n">
-        <v>342.33</v>
-      </c>
-      <c r="AU14" s="2" t="n">
-        <v>113.3</v>
-      </c>
-      <c r="AV14" s="2" t="n">
-        <v>156.554</v>
-      </c>
-      <c r="AW14" s="2" t="n">
-        <v>230.808</v>
-      </c>
-      <c r="AX14" s="2" t="n">
-        <v>264.695</v>
-      </c>
-      <c r="AY14" s="2" t="n">
-        <v>172.232</v>
-      </c>
-      <c r="AZ14" s="2" t="n">
-        <v>735.4</v>
-      </c>
-      <c r="BA14" s="2" t="n">
-        <v>693.1</v>
-      </c>
-      <c r="BB14" s="2" t="n">
-        <v>0.5143</v>
-      </c>
-      <c r="BC14" s="2" t="n">
-        <v>0.4481</v>
-      </c>
-      <c r="BD14" s="2" t="n">
-        <v>0.508</v>
-      </c>
-      <c r="BE14" s="2" t="n">
-        <v>0.4379</v>
-      </c>
-      <c r="BF14" s="2" t="n">
-        <v>0.5061</v>
-      </c>
-      <c r="BG14" s="2" t="n">
-        <v>0.4326</v>
-      </c>
-      <c r="BH14" s="2" t="n">
-        <v>0.9295</v>
+        <v>0.9441000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added calculations of finding true b/t
</commit_message>
<xml_diff>
--- a/export/Приложение_А.xlsx
+++ b/export/Приложение_А.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH12"/>
+  <dimension ref="A1:BH14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -800,28 +800,28 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.7764</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.7196</v>
+        <v>0.6266</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.5546</v>
+        <v>0.427</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.45</v>
+        <v>0.4884</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>172.9</v>
+        <v>170.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.8575</v>
+        <v>0.8612</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.2511</v>
+        <v>0.2423</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>0.99</v>
@@ -830,151 +830,151 @@
         <v>0.5</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>58.773</v>
+        <v>62.58</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>37067.556</v>
+        <v>29616.784</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>36696.88</v>
+        <v>29320.616</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>31468.57</v>
+        <v>25250.985</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>324.4</v>
+        <v>317.1</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>100.713</v>
+        <v>100.658</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>144.49</v>
+        <v>134.86</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>1.4347</v>
+        <v>1.3398</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>310.726</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>1.013</v>
+        <v>1.031</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>0.8434</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.2728</v>
+        <v>0.2534</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>0.6506999999999999</v>
+        <v>0.619</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>0.3351</v>
+        <v>0.3334</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.6036</v>
+        <v>0.5785</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>0.2655</v>
+        <v>0.278</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>0.732</v>
+        <v>0.6425999999999999</v>
       </c>
       <c r="AD2" s="2" t="n">
-        <v>0.8763</v>
+        <v>0.8405</v>
       </c>
       <c r="AE2" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AF2" s="2" t="n">
-        <v>0.2814</v>
+        <v>0.2605</v>
       </c>
       <c r="AG2" s="2" t="n">
-        <v>56.99</v>
+        <v>60.867</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>0.434</v>
+        <v>0.4685</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>166.8</v>
+        <v>163.8</v>
       </c>
       <c r="AJ2" s="2" t="n">
         <v>6</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>1.325</v>
+        <v>1.282</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>0.8598</v>
+        <v>0.8238</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>0.4344</v>
+        <v>0.4712</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.5596</v>
+        <v>0.5424</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>37.819</v>
+        <v>40.985</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>38.264</v>
+        <v>41.417</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>55.351</v>
+        <v>59.158</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>17.087</v>
+        <v>17.74</v>
       </c>
       <c r="AS2" s="2" t="n">
-        <v>19.171</v>
+        <v>19.882</v>
       </c>
       <c r="AT2" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>166.9</v>
+        <v>164.7</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>202.195</v>
+        <v>192.354</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>272.192</v>
+        <v>251.189</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>279.196</v>
+        <v>258.102</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>202.883</v>
+        <v>191.879</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>324.4</v>
+        <v>317.1</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>267.7</v>
+        <v>269.6</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>0.9546</v>
+        <v>0.893</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>0.8963</v>
+        <v>0.8425</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>0.8509</v>
+        <v>0.7838000000000001</v>
       </c>
       <c r="BE2" s="2" t="n">
-        <v>0.8004</v>
+        <v>0.741</v>
       </c>
       <c r="BF2" s="2" t="n">
-        <v>0.8038</v>
+        <v>0.7277</v>
       </c>
       <c r="BG2" s="2" t="n">
-        <v>0.7658</v>
+        <v>0.6958</v>
       </c>
       <c r="BH2" s="2" t="n">
-        <v>0.6909</v>
+        <v>0.5954</v>
       </c>
     </row>
     <row r="3">
@@ -982,181 +982,181 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.7764</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.7477</v>
+        <v>0.652</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.6245000000000001</v>
+        <v>0.4975</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.434</v>
+        <v>0.4685</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>166.8</v>
+        <v>163.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.8653</v>
+        <v>0.8716</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.2747</v>
+        <v>0.2685</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.985</v>
+        <v>0.986</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>0.7318</v>
+        <v>0.6407</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>57.045</v>
+        <v>60.964</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>40557.559</v>
+        <v>32814.186</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>39949.195</v>
+        <v>32349.318</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>34567.937</v>
+        <v>28197.116</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>364.1</v>
+        <v>349.2</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>144.49</v>
+        <v>134.86</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>205.536</v>
+        <v>181.404</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>1.4225</v>
+        <v>1.3451</v>
       </c>
       <c r="U3" s="2" t="n">
-        <v>329.763</v>
+        <v>326.03</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>1.326</v>
+        <v>1.284</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>0.8762</v>
+        <v>0.8398</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.2814</v>
+        <v>0.2601</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>0.6026</v>
+        <v>0.5746</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>0.2656</v>
+        <v>0.2791</v>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.5548</v>
+        <v>0.5333</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>0.2126</v>
+        <v>0.2329</v>
       </c>
       <c r="AC3" s="2" t="n">
-        <v>0.7926</v>
+        <v>0.7128</v>
       </c>
       <c r="AD3" s="2" t="n">
-        <v>0.9023</v>
+        <v>0.8683</v>
       </c>
       <c r="AE3" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AF3" s="2" t="n">
-        <v>0.2867</v>
+        <v>0.2659</v>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>55.853</v>
+        <v>59.66</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>0.4231</v>
+        <v>0.4549</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>162.6</v>
+        <v>159</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>6.4</v>
+        <v>6.333</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>1.722</v>
+        <v>1.601</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>0.8893</v>
+        <v>0.8541</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>0.4173</v>
+        <v>0.4504</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.5862000000000001</v>
+        <v>0.5701000000000001</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>35.45</v>
+        <v>38.309</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>36.113</v>
+        <v>38.941</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>54.012</v>
+        <v>57.763</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>17.899</v>
+        <v>18.822</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>20.403</v>
+        <v>21.351</v>
       </c>
       <c r="AT3" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>160.4</v>
+        <v>157.4</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>198.727</v>
+        <v>187.326</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>276.474</v>
+        <v>253.988</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>282.931</v>
+        <v>260.586</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>198.176</v>
+        <v>186.144</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>364.1</v>
+        <v>349.2</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>304.9</v>
+        <v>299.7</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>0.8845</v>
+        <v>0.8361</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>0.8349</v>
+        <v>0.7914</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>0.8082</v>
+        <v>0.7507</v>
       </c>
       <c r="BE3" s="2" t="n">
-        <v>0.7639</v>
+        <v>0.7115</v>
       </c>
       <c r="BF3" s="2" t="n">
-        <v>0.7744</v>
+        <v>0.7079</v>
       </c>
       <c r="BG3" s="2" t="n">
-        <v>0.7395</v>
+        <v>0.6777</v>
       </c>
       <c r="BH3" s="2" t="n">
-        <v>0.7634</v>
+        <v>0.678</v>
       </c>
     </row>
     <row r="4">
@@ -1164,181 +1164,181 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.7764</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.7708</v>
+        <v>0.675</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.6783</v>
+        <v>0.5554</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.4231</v>
+        <v>0.4549</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>162.6</v>
+        <v>159</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.8726</v>
+        <v>0.8804</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.2967</v>
+        <v>0.2922</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.98</v>
+        <v>0.982</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.7154</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>55.812</v>
+        <v>59.62</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>43805.585</v>
+        <v>35711.611</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>42929.473</v>
+        <v>35056.898</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>37458.473</v>
+        <v>30864.024</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>406.5</v>
+        <v>383.9</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>205.536</v>
+        <v>181.404</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>289.039</v>
+        <v>243.601</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>1.4063</v>
+        <v>1.3429</v>
       </c>
       <c r="U4" s="2" t="n">
-        <v>349.224</v>
+        <v>342.068</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>1.715</v>
+        <v>1.596</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>0.9033</v>
+        <v>0.8694</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>0.2874</v>
+        <v>0.2667</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>0.5627</v>
+        <v>0.5389</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>0.2105</v>
+        <v>0.2312</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.5208</v>
+        <v>0.5023</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>0.171</v>
+        <v>0.1943</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>0.8372000000000001</v>
+        <v>0.7678</v>
       </c>
       <c r="AD4" s="2" t="n">
-        <v>0.9222</v>
+        <v>0.8915</v>
       </c>
       <c r="AE4" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AF4" s="2" t="n">
-        <v>0.2982</v>
+        <v>0.2788</v>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>54.181</v>
+        <v>57.783</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>0.4135</v>
+        <v>0.443</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>158.9</v>
+        <v>154.9</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>6.8</v>
+        <v>6.667</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>2.203</v>
+        <v>1.983</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>0.9127</v>
+        <v>0.8804999999999999</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>0.4054</v>
+        <v>0.4358</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.6095</v>
+        <v>0.5952</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>33.628</v>
+        <v>36.214</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>34.487</v>
+        <v>37.043</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>53.204</v>
+        <v>56.792</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>18.717</v>
+        <v>19.749</v>
       </c>
       <c r="AS4" s="2" t="n">
-        <v>20.554</v>
+        <v>21.569</v>
       </c>
       <c r="AT4" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>155.8</v>
+        <v>152.4</v>
       </c>
       <c r="AV4" s="2" t="n">
-        <v>196.519</v>
+        <v>184.349</v>
       </c>
       <c r="AW4" s="2" t="n">
-        <v>281.26</v>
+        <v>257.9</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>287.098</v>
+        <v>264</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>194.512</v>
+        <v>182.11</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>406.5</v>
+        <v>383.9</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>345</v>
+        <v>332.4</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>0.8262</v>
+        <v>0.7874</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>0.7841</v>
+        <v>0.7484</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>0.7715</v>
+        <v>0.7225</v>
       </c>
       <c r="BE4" s="2" t="n">
-        <v>0.7329</v>
+        <v>0.6872</v>
       </c>
       <c r="BF4" s="2" t="n">
-        <v>0.746</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="BG4" s="2" t="n">
-        <v>0.714</v>
+        <v>0.6606</v>
       </c>
       <c r="BH4" s="2" t="n">
-        <v>0.8174</v>
+        <v>0.7433</v>
       </c>
     </row>
     <row r="5">
@@ -1346,181 +1346,181 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.7764</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.7879</v>
+        <v>0.6933</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.7166</v>
+        <v>0.5988</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.4135</v>
+        <v>0.443</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>158.9</v>
+        <v>154.9</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.8692</v>
+        <v>0.878</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.3005</v>
+        <v>0.2977</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0.975</v>
+        <v>0.978</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0.8399</v>
+        <v>0.7712</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>54.13</v>
+        <v>57.722</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>44357.527</v>
+        <v>36381.104</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>43248.589</v>
+        <v>35562.529</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>37592.953</v>
+        <v>31225.552</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>449</v>
+        <v>419</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>289.039</v>
+        <v>243.601</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>393.286</v>
+        <v>319.817</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>1.3607</v>
+        <v>1.3129</v>
       </c>
       <c r="U5" s="2" t="n">
-        <v>368.861</v>
+        <v>358.555</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>2.192</v>
+        <v>1.975</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>0.9234</v>
+        <v>0.893</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>0.299</v>
+        <v>0.2798</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>0.5316</v>
+        <v>0.5109</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>0.1685</v>
+        <v>0.1919</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.4909</v>
+        <v>0.4748</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>0.1407</v>
+        <v>0.1645</v>
       </c>
       <c r="AC5" s="2" t="n">
-        <v>0.8683</v>
+        <v>0.8078</v>
       </c>
       <c r="AD5" s="2" t="n">
-        <v>0.9364</v>
+        <v>0.909</v>
       </c>
       <c r="AE5" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AF5" s="2" t="n">
-        <v>0.306</v>
+        <v>0.2881</v>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>52.892</v>
+        <v>56.284</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>0.4047</v>
+        <v>0.4321</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>155.5</v>
+        <v>151.1</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>2.75</v>
+        <v>2.413</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>0.9298999999999999</v>
+        <v>0.901</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>0.3948</v>
+        <v>0.423</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.62</v>
+        <v>0.6077</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>32.486</v>
+        <v>34.839</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>33.515</v>
+        <v>35.848</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>51.867</v>
+        <v>55.264</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>18.352</v>
+        <v>19.416</v>
       </c>
       <c r="AS5" s="2" t="n">
-        <v>20.406</v>
+        <v>21.445</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>151.7</v>
+        <v>147.9</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>196.07</v>
+        <v>183.184</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>282.419</v>
+        <v>258.853</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>287.751</v>
+        <v>264.457</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>192.839</v>
+        <v>179.944</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>449</v>
+        <v>419</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>387.6</v>
+        <v>367.4</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>0.7696</v>
+        <v>0.7379</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>0.7348</v>
+        <v>0.7048</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>0.7302</v>
+        <v>0.6889</v>
       </c>
       <c r="BE5" s="2" t="n">
-        <v>0.6977</v>
+        <v>0.6584</v>
       </c>
       <c r="BF5" s="2" t="n">
-        <v>0.7103</v>
+        <v>0.662</v>
       </c>
       <c r="BG5" s="2" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.6361</v>
       </c>
       <c r="BH5" s="2" t="n">
-        <v>0.8554</v>
+        <v>0.7913</v>
       </c>
     </row>
     <row r="6">
@@ -1528,181 +1528,181 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.7764</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8001</v>
+        <v>0.707</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.7432</v>
+        <v>0.63</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.4047</v>
+        <v>0.4321</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>155.5</v>
+        <v>151.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.8658</v>
+        <v>0.8753</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0.3038</v>
+        <v>0.3025</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.97</v>
+        <v>0.973</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0.871</v>
+        <v>0.8114</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>52.828</v>
+        <v>56.201</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>44843.01</v>
+        <v>36967.636</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>43497.72</v>
+        <v>35981.832</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>37659.32</v>
+        <v>31493.976</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>491.5</v>
+        <v>454.3</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>393.286</v>
+        <v>319.817</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>520.6130000000001</v>
+        <v>411.612</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>1.3238</v>
+        <v>1.287</v>
       </c>
       <c r="U6" s="2" t="n">
-        <v>387.471</v>
+        <v>374.432</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>2.734</v>
+        <v>2.402</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>0.9377</v>
+        <v>0.9106</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>0.3069</v>
+        <v>0.2892</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>0.5037</v>
+        <v>0.4855</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>0.138</v>
+        <v>0.1617</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.4643</v>
+        <v>0.4501</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>0.1181</v>
+        <v>0.1412</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>0.8908</v>
+        <v>0.8377</v>
       </c>
       <c r="AD6" s="2" t="n">
-        <v>0.947</v>
+        <v>0.9224</v>
       </c>
       <c r="AE6" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AF6" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.2949</v>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>51.833</v>
+        <v>55.026</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>0.3965</v>
+        <v>0.4218</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>152.3</v>
+        <v>147.5</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>7.6</v>
+        <v>7.333</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>3.361</v>
+        <v>2.892</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>0.9423</v>
+        <v>0.9165</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>0.385</v>
+        <v>0.4111</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.6277</v>
+        <v>0.6173999999999999</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>31.519</v>
+        <v>33.659</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>32.684</v>
+        <v>34.812</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>50.741</v>
+        <v>53.957</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>18.057</v>
+        <v>19.145</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>20.314</v>
+        <v>21.367</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>147.9</v>
+        <v>143.7</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>195.16</v>
+        <v>181.773</v>
       </c>
       <c r="AW6" s="2" t="n">
-        <v>282.929</v>
+        <v>259.308</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>287.977</v>
+        <v>264.593</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>191.024</v>
+        <v>177.745</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>491.5</v>
+        <v>454.3</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>430.4</v>
+        <v>402.8</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>0.7239</v>
+        <v>0.697</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>0.6941000000000001</v>
+        <v>0.6682</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>0.6944</v>
+        <v>0.6589</v>
       </c>
       <c r="BE6" s="2" t="n">
-        <v>0.6662</v>
+        <v>0.6319</v>
       </c>
       <c r="BF6" s="2" t="n">
-        <v>0.6784</v>
+        <v>0.6368</v>
       </c>
       <c r="BG6" s="2" t="n">
-        <v>0.6531</v>
+        <v>0.6131</v>
       </c>
       <c r="BH6" s="2" t="n">
-        <v>0.8823</v>
+        <v>0.8264</v>
       </c>
     </row>
     <row r="7">
@@ -1710,181 +1710,181 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.7764</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8091</v>
+        <v>0.7175</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.7624</v>
+        <v>0.6533</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.3965</v>
+        <v>0.4218</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>152.3</v>
+        <v>147.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0.8622</v>
+        <v>0.8721</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.3067</v>
+        <v>0.3068</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0.965</v>
+        <v>0.969</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>0.8935</v>
+        <v>0.8414</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>51.764</v>
+        <v>54.934</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>45280.09</v>
+        <v>37493.555</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>43695.286</v>
+        <v>36337.504</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>37673.688</v>
+        <v>31691.342</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>533.9</v>
+        <v>489.8</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>520.6130000000001</v>
+        <v>411.612</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>673.3339999999999</v>
+        <v>520.55</v>
       </c>
       <c r="T7" s="2" t="n">
-        <v>1.2933</v>
+        <v>1.2647</v>
       </c>
       <c r="U7" s="2" t="n">
-        <v>405.144</v>
+        <v>389.716</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>3.342</v>
+        <v>2.878</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>0.9483</v>
+        <v>0.9241</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.3124</v>
+        <v>0.2961</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.4787</v>
+        <v>0.4623</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>0.1153</v>
+        <v>0.1383</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>0.4406</v>
+        <v>0.4276</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>0.1007</v>
+        <v>0.1227</v>
       </c>
       <c r="AC7" s="2" t="n">
-        <v>0.9077</v>
+        <v>0.8607</v>
       </c>
       <c r="AD7" s="2" t="n">
-        <v>0.955</v>
+        <v>0.9329</v>
       </c>
       <c r="AE7" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AF7" s="2" t="n">
-        <v>0.3155</v>
+        <v>0.3</v>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>50.927</v>
+        <v>53.937</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>0.3886</v>
+        <v>0.412</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>149.3</v>
+        <v>144.1</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>8</v>
+        <v>7.667</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>4.039</v>
+        <v>3.421</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>0.9516</v>
+        <v>0.9285</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>0.3757</v>
+        <v>0.3999</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>0.6336000000000001</v>
+        <v>0.625</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>30.663</v>
+        <v>32.61</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>31.945</v>
+        <v>33.887</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>49.752</v>
+        <v>52.803</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>17.806</v>
+        <v>18.916</v>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>20.263</v>
+        <v>21.327</v>
       </c>
       <c r="AT7" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>144.3</v>
+        <v>139.8</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>193.947</v>
+        <v>180.17</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>283.023</v>
+        <v>259.412</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>287.916</v>
+        <v>264.489</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>189.111</v>
+        <v>175.504</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>533.9</v>
+        <v>489.8</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>473.3</v>
+        <v>438.5</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>0.6859</v>
+        <v>0.6624</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>0.6597</v>
+        <v>0.6368</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>0.663</v>
+        <v>0.632</v>
       </c>
       <c r="BE7" s="2" t="n">
-        <v>0.6381</v>
+        <v>0.6078</v>
       </c>
       <c r="BF7" s="2" t="n">
-        <v>0.6499</v>
+        <v>0.6135</v>
       </c>
       <c r="BG7" s="2" t="n">
-        <v>0.627</v>
+        <v>0.5917</v>
       </c>
       <c r="BH7" s="2" t="n">
-        <v>0.902</v>
+        <v>0.8529</v>
       </c>
     </row>
     <row r="8">
@@ -1892,181 +1892,181 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.7764</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8159</v>
+        <v>0.7257</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.7768</v>
+        <v>0.6711</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>384.23</v>
+        <v>349.61</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.3886</v>
+        <v>0.412</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>149.3</v>
+        <v>144.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.8585</v>
+        <v>0.8687</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.3094</v>
+        <v>0.3107</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.96</v>
+        <v>0.965</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0.9104</v>
+        <v>0.8643999999999999</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>50.856</v>
+        <v>53.839</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>45678.947</v>
+        <v>37971.482</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>43851.789</v>
+        <v>36642.481</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>37645.531</v>
+        <v>31830.509</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>576.1</v>
+        <v>525.3</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>673.3339999999999</v>
+        <v>520.55</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>853.73</v>
+        <v>648.178</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>1.2679</v>
+        <v>1.2452</v>
       </c>
       <c r="U8" s="2" t="n">
-        <v>421.963</v>
+        <v>404.436</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>4.015</v>
+        <v>3.404</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>0.9562</v>
+        <v>0.9347</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0.3163</v>
+        <v>0.3011</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>0.4563</v>
+        <v>0.4412</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>0.0979</v>
+        <v>0.1197</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>0.4192</v>
+        <v>0.4071</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>0.0871</v>
+        <v>0.1078</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>0.9191</v>
+        <v>0.8788</v>
       </c>
       <c r="AD8" s="2" t="n">
-        <v>0.9604</v>
+        <v>0.9413</v>
       </c>
       <c r="AE8" s="2" t="n">
-        <v>379.86</v>
+        <v>349.61</v>
       </c>
       <c r="AF8" s="2" t="n">
-        <v>0.3178</v>
+        <v>0.3038</v>
       </c>
       <c r="AG8" s="2" t="n">
-        <v>50.125</v>
+        <v>52.967</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>0.3811</v>
+        <v>0.4027</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>144.8</v>
+        <v>140.8</v>
       </c>
       <c r="AJ8" s="2" t="n">
-        <v>8.4</v>
+        <v>8</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>4.784</v>
+        <v>4.001</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>0.9583</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>0.3668</v>
+        <v>0.3892</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>0.6385</v>
+        <v>0.6313</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>29.874</v>
+        <v>31.653</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>31.272</v>
+        <v>33.04</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>48.913</v>
+        <v>51.756</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>17.641</v>
+        <v>18.715</v>
       </c>
       <c r="AS8" s="2" t="n">
-        <v>20.251</v>
+        <v>21.314</v>
       </c>
       <c r="AT8" s="2" t="n">
-        <v>382.04</v>
+        <v>349.61</v>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>140.9</v>
+        <v>136.1</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>192.539</v>
+        <v>178.428</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>282.93</v>
+        <v>259.266</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>287.664</v>
+        <v>264.212</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>186.976</v>
+        <v>173.236</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>576.1</v>
+        <v>525.3</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>516.1</v>
+        <v>474.4</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>0.6466</v>
+        <v>0.6325</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>0.6253</v>
+        <v>0.6095</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>0.6354</v>
+        <v>0.6077</v>
       </c>
       <c r="BE8" s="2" t="n">
-        <v>0.6131</v>
+        <v>0.5857</v>
       </c>
       <c r="BF8" s="2" t="n">
-        <v>0.6173</v>
+        <v>0.592</v>
       </c>
       <c r="BG8" s="2" t="n">
-        <v>0.5982</v>
+        <v>0.5718</v>
       </c>
       <c r="BH8" s="2" t="n">
-        <v>0.9156</v>
+        <v>0.8734</v>
       </c>
     </row>
     <row r="9">
@@ -2074,181 +2074,181 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.8436</v>
+        <v>0.7764</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8109</v>
+        <v>0.7322</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.7768</v>
+        <v>0.6852</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>379.86</v>
+        <v>349.61</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.3811</v>
+        <v>0.4027</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>144.8</v>
+        <v>140.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.8546</v>
+        <v>0.8649</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.3119</v>
+        <v>0.3142</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.955</v>
+        <v>0.961</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>0.9209000000000001</v>
+        <v>0.8825</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>50.126</v>
+        <v>52.866</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>46046.107</v>
+        <v>38409.522</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>43974.032</v>
+        <v>36905.15</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>37581.17</v>
+        <v>31920.004</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>618</v>
+        <v>560.9</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>853.73</v>
+        <v>648.178</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>1064.033</v>
+        <v>796.019</v>
       </c>
       <c r="T9" s="2" t="n">
-        <v>1.2463</v>
+        <v>1.2281</v>
       </c>
       <c r="U9" s="2" t="n">
-        <v>438.003</v>
+        <v>418.62</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>4.764</v>
+        <v>3.98</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>0.9612000000000001</v>
+        <v>0.9431</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>0.3184</v>
+        <v>0.3049</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>0.4307</v>
+        <v>0.4218</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.1047</v>
       </c>
       <c r="AA9" s="2" t="n">
-        <v>0.3945</v>
+        <v>0.3884</v>
       </c>
       <c r="AB9" s="2" t="n">
-        <v>0.077</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="AC9" s="2" t="n">
-        <v>0.9275</v>
+        <v>0.8932</v>
       </c>
       <c r="AD9" s="2" t="n">
-        <v>0.9644</v>
+        <v>0.9481000000000001</v>
       </c>
       <c r="AE9" s="2" t="n">
-        <v>376.33</v>
+        <v>349.61</v>
       </c>
       <c r="AF9" s="2" t="n">
-        <v>0.3193</v>
+        <v>0.3066</v>
       </c>
       <c r="AG9" s="2" t="n">
-        <v>49.498</v>
+        <v>52.083</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>0.3739</v>
+        <v>0.3937</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>140.7</v>
+        <v>137.6</v>
       </c>
       <c r="AJ9" s="2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.333</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>5.606</v>
+        <v>4.631</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>0.9628</v>
+        <v>0.9456</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>0.358</v>
+        <v>0.3789</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>0.6418</v>
+        <v>0.6364</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>29.15</v>
+        <v>30.764</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>30.662</v>
+        <v>32.253</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>48.113</v>
+        <v>50.784</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>17.451</v>
+        <v>18.531</v>
       </c>
       <c r="AS9" s="2" t="n">
-        <v>20.348</v>
+        <v>21.319</v>
       </c>
       <c r="AT9" s="2" t="n">
-        <v>378.1</v>
+        <v>349.61</v>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>136</v>
+        <v>132.5</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>188.642</v>
+        <v>176.593</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>279.148</v>
+        <v>258.944</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>283.886</v>
+        <v>263.808</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>182.647</v>
+        <v>170.955</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>618</v>
+        <v>560.9</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>559.1</v>
+        <v>510.3</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>0.6156</v>
+        <v>0.6064000000000001</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>0.5961</v>
+        <v>0.5853</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>0.6034</v>
+        <v>0.5858</v>
       </c>
       <c r="BE9" s="2" t="n">
-        <v>0.583</v>
+        <v>0.5656</v>
       </c>
       <c r="BF9" s="2" t="n">
-        <v>0.591</v>
+        <v>0.5723</v>
       </c>
       <c r="BG9" s="2" t="n">
-        <v>0.5732</v>
+        <v>0.5534</v>
       </c>
       <c r="BH9" s="2" t="n">
-        <v>0.9251</v>
+        <v>0.8897</v>
       </c>
     </row>
     <row r="10">
@@ -2256,181 +2256,181 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.8357</v>
+        <v>0.7764</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8068</v>
+        <v>0.7375</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.7768</v>
+        <v>0.6964</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>376.33</v>
+        <v>349.61</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.3739</v>
+        <v>0.3937</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>140.7</v>
+        <v>137.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.8506</v>
+        <v>0.8609</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.3142</v>
+        <v>0.3176</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.95</v>
+        <v>0.957</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0.9295</v>
+        <v>0.8969</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>49.443</v>
+        <v>51.981</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>46386.108</v>
+        <v>38813.315</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>44066.802</v>
+        <v>37131.405</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>37485.176</v>
+        <v>31965.961</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>659.6</v>
+        <v>596.4</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>1064.033</v>
+        <v>796.019</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>1306.42</v>
+        <v>965.558</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>1.2278</v>
+        <v>1.213</v>
       </c>
       <c r="U10" s="2" t="n">
-        <v>453.334</v>
+        <v>432.3</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>5.579</v>
+        <v>4.606</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0.9654</v>
+        <v>0.9499</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>0.32</v>
+        <v>0.3078</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>0.4085</v>
+        <v>0.4041</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>0.0746</v>
+        <v>0.0926</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>0.3675</v>
+        <v>0.3711</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.0857</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>0.9346</v>
+        <v>0.905</v>
       </c>
       <c r="AD10" s="2" t="n">
-        <v>0.9679</v>
+        <v>0.9537</v>
       </c>
       <c r="AE10" s="2" t="n">
-        <v>373.38</v>
+        <v>349.61</v>
       </c>
       <c r="AF10" s="2" t="n">
-        <v>0.3093</v>
+        <v>0.3088</v>
       </c>
       <c r="AG10" s="2" t="n">
-        <v>49.863</v>
+        <v>51.262</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>0.3668</v>
+        <v>0.3849</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>137</v>
+        <v>134.6</v>
       </c>
       <c r="AJ10" s="2" t="n">
-        <v>9.199999999999999</v>
+        <v>8.667</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>6.505</v>
+        <v>5.312</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>0.9666</v>
+        <v>0.9518</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>0.3494</v>
+        <v>0.3689</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>0.6446</v>
+        <v>0.6408</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>28.461</v>
+        <v>29.927</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>30.082</v>
+        <v>31.513</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>47.337</v>
+        <v>49.868</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>17.255</v>
+        <v>18.355</v>
       </c>
       <c r="AS10" s="2" t="n">
-        <v>21.402</v>
+        <v>21.336</v>
       </c>
       <c r="AT10" s="2" t="n">
-        <v>374.86</v>
+        <v>349.61</v>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>131.5</v>
+        <v>129</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>185.188</v>
+        <v>174.698</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>275.933</v>
+        <v>258.496</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>280.704</v>
+        <v>263.311</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>178.825</v>
+        <v>168.675</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>659.6</v>
+        <v>596.4</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>601.8</v>
+        <v>546.3</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.5889</v>
+        <v>0.5832000000000001</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>0.5709</v>
+        <v>0.5638</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>0.5760999999999999</v>
+        <v>0.5659</v>
       </c>
       <c r="BE10" s="2" t="n">
-        <v>0.5571</v>
+        <v>0.5472</v>
       </c>
       <c r="BF10" s="2" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.5542</v>
       </c>
       <c r="BG10" s="2" t="n">
-        <v>0.5512</v>
+        <v>0.5364</v>
       </c>
       <c r="BH10" s="2" t="n">
-        <v>0.9331</v>
+        <v>0.9028</v>
       </c>
     </row>
     <row r="11">
@@ -2438,181 +2438,181 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.8292</v>
+        <v>0.7764</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8034</v>
+        <v>0.7418</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.7768</v>
+        <v>0.7055</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>373.38</v>
+        <v>349.61</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.3668</v>
+        <v>0.3849</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>137</v>
+        <v>134.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.8364</v>
+        <v>0.8566</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.3005</v>
+        <v>0.3206</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.945</v>
+        <v>0.952</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0.9368</v>
+        <v>0.9087</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>49.8</v>
+        <v>51.16</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>44367.168</v>
+        <v>39187.011</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>41926.974</v>
+        <v>37325.628</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>35067.072</v>
+        <v>31973.049</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>698.9</v>
+        <v>631.8</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>1306.42</v>
+        <v>965.558</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>1564.88</v>
+        <v>1158.231</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>1.1978</v>
+        <v>1.1995</v>
       </c>
       <c r="U11" s="2" t="n">
-        <v>468.019</v>
+        <v>445.507</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>6.472</v>
+        <v>5.283</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.9689</v>
+        <v>0.9554</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.31</v>
+        <v>0.3099</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>0.3832</v>
+        <v>0.3878</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>0.06610000000000001</v>
+        <v>0.0825</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>0.3393</v>
+        <v>0.3552</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>0.0621</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="AC11" s="2" t="n">
-        <v>0.9403</v>
+        <v>0.9147</v>
       </c>
       <c r="AD11" s="2" t="n">
-        <v>0.9706</v>
+        <v>0.9583</v>
       </c>
       <c r="AE11" s="2" t="n">
-        <v>371.07</v>
+        <v>349.61</v>
       </c>
       <c r="AF11" s="2" t="n">
-        <v>0.2892</v>
+        <v>0.3104</v>
       </c>
       <c r="AG11" s="2" t="n">
-        <v>51.23</v>
+        <v>50.488</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>0.36</v>
+        <v>0.3764</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>133.6</v>
+        <v>131.6</v>
       </c>
       <c r="AJ11" s="2" t="n">
-        <v>9.6</v>
+        <v>9</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>7.417</v>
+        <v>6.045</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>0.9698</v>
+        <v>0.9569</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>0.3411</v>
+        <v>0.3592</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>0.6196</v>
+        <v>0.6445</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>28.834</v>
+        <v>29.13</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>29.106</v>
+        <v>30.808</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>44.255</v>
+        <v>48.99</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>15.149</v>
+        <v>18.182</v>
       </c>
       <c r="AS11" s="2" t="n">
-        <v>22.396</v>
+        <v>21.359</v>
       </c>
       <c r="AT11" s="2" t="n">
-        <v>372.23</v>
+        <v>349.61</v>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>127.4</v>
+        <v>125.6</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>179.329</v>
+        <v>172.77</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>264.105</v>
+        <v>257.958</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>281.589</v>
+        <v>262.748</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>182.519</v>
+        <v>166.407</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>698.9</v>
+        <v>631.8</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>644.6</v>
+        <v>582.2</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>0.5707</v>
+        <v>0.5625</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>0.5302</v>
+        <v>0.5444</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>0.5594</v>
+        <v>0.5477</v>
       </c>
       <c r="BE11" s="2" t="n">
-        <v>0.5167</v>
+        <v>0.5303</v>
       </c>
       <c r="BF11" s="2" t="n">
-        <v>0.5567</v>
+        <v>0.5375</v>
       </c>
       <c r="BG11" s="2" t="n">
-        <v>0.5141</v>
+        <v>0.5207000000000001</v>
       </c>
       <c r="BH11" s="2" t="n">
-        <v>0.9397</v>
+        <v>0.9135</v>
       </c>
     </row>
     <row r="12">
@@ -2620,181 +2620,545 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.8241000000000001</v>
+        <v>0.7764</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8008</v>
+        <v>0.7454</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.7768</v>
+        <v>0.713</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>371.07</v>
+        <v>349.61</v>
       </c>
       <c r="F12" s="2" t="n">
+        <v>0.3764</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>131.6</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.8521</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.3234</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0.948</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0.9183</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>50.385</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>39533.793</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>37491.214</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>31944.972</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>667.1</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>1158.231</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>1375.412</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>1.1875</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>458.269</v>
+      </c>
+      <c r="V12" s="2" t="n">
+        <v>6.011</v>
+      </c>
+      <c r="W12" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="X12" s="2" t="n">
+        <v>0.3116</v>
+      </c>
+      <c r="Y12" s="2" t="n">
+        <v>0.3728</v>
+      </c>
+      <c r="Z12" s="2" t="n">
+        <v>0.0742</v>
+      </c>
+      <c r="AA12" s="2" t="n">
+        <v>0.3355</v>
+      </c>
+      <c r="AB12" s="2" t="n">
+        <v>0.0702</v>
+      </c>
+      <c r="AC12" s="2" t="n">
+        <v>0.9222</v>
+      </c>
+      <c r="AD12" s="2" t="n">
+        <v>0.9619</v>
+      </c>
+      <c r="AE12" s="2" t="n">
+        <v>347.06</v>
+      </c>
+      <c r="AF12" s="2" t="n">
+        <v>0.3007</v>
+      </c>
+      <c r="AG12" s="2" t="n">
+        <v>50.739</v>
+      </c>
+      <c r="AH12" s="2" t="n">
+        <v>0.3681</v>
+      </c>
+      <c r="AI12" s="2" t="n">
+        <v>127.8</v>
+      </c>
+      <c r="AJ12" s="2" t="n">
+        <v>9.333</v>
+      </c>
+      <c r="AK12" s="2" t="n">
+        <v>6.837</v>
+      </c>
+      <c r="AL12" s="2" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="AM12" s="2" t="n">
+        <v>0.3497</v>
+      </c>
+      <c r="AN12" s="2" t="n">
+        <v>0.6478</v>
+      </c>
+      <c r="AO12" s="2" t="n">
+        <v>28.361</v>
+      </c>
+      <c r="AP12" s="2" t="n">
+        <v>30.133</v>
+      </c>
+      <c r="AQ12" s="2" t="n">
+        <v>48.161</v>
+      </c>
+      <c r="AR12" s="2" t="n">
+        <v>18.027</v>
+      </c>
+      <c r="AS12" s="2" t="n">
+        <v>22.379</v>
+      </c>
+      <c r="AT12" s="2" t="n">
+        <v>348.34</v>
+      </c>
+      <c r="AU12" s="2" t="n">
+        <v>122.3</v>
+      </c>
+      <c r="AV12" s="2" t="n">
+        <v>170.827</v>
+      </c>
+      <c r="AW12" s="2" t="n">
+        <v>257.385</v>
+      </c>
+      <c r="AX12" s="2" t="n">
+        <v>262.136</v>
+      </c>
+      <c r="AY12" s="2" t="n">
+        <v>164.107</v>
+      </c>
+      <c r="AZ12" s="2" t="n">
+        <v>667.1</v>
+      </c>
+      <c r="BA12" s="2" t="n">
+        <v>618.1</v>
+      </c>
+      <c r="BB12" s="2" t="n">
+        <v>0.5403</v>
+      </c>
+      <c r="BC12" s="2" t="n">
+        <v>0.5244</v>
+      </c>
+      <c r="BD12" s="2" t="n">
+        <v>0.5312</v>
+      </c>
+      <c r="BE12" s="2" t="n">
+        <v>0.5148</v>
+      </c>
+      <c r="BF12" s="2" t="n">
+        <v>0.5184</v>
+      </c>
+      <c r="BG12" s="2" t="n">
+        <v>0.5034</v>
+      </c>
+      <c r="BH12" s="2" t="n">
+        <v>0.9217</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0.7707000000000001</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0.7423999999999999</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>0.713</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>347.06</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.3681</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>127.8</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.8371</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0.3098</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>0.9251</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>50.675</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>37863.373</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>35749.334</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>29927.042</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>700.5</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>1375.412</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>1602.645</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>1.1652</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>470.614</v>
+      </c>
+      <c r="V13" s="2" t="n">
+        <v>6.806</v>
+      </c>
+      <c r="W13" s="2" t="n">
+        <v>0.9633</v>
+      </c>
+      <c r="X13" s="2" t="n">
+        <v>0.3016</v>
+      </c>
+      <c r="Y13" s="2" t="n">
+        <v>0.3509</v>
+      </c>
+      <c r="Z13" s="2" t="n">
+        <v>0.0673</v>
+      </c>
+      <c r="AA13" s="2" t="n">
+        <v>0.3106</v>
+      </c>
+      <c r="AB13" s="2" t="n">
+        <v>0.06510000000000001</v>
+      </c>
+      <c r="AC13" s="2" t="n">
+        <v>0.9273</v>
+      </c>
+      <c r="AD13" s="2" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="AE13" s="2" t="n">
+        <v>345.06</v>
+      </c>
+      <c r="AF13" s="2" t="n">
+        <v>0.2806</v>
+      </c>
+      <c r="AG13" s="2" t="n">
+        <v>52.065</v>
+      </c>
+      <c r="AH13" s="2" t="n">
         <v>0.36</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>133.6</v>
-      </c>
-      <c r="H12" s="2" t="n">
+      <c r="AI13" s="2" t="n">
+        <v>124.2</v>
+      </c>
+      <c r="AJ13" s="2" t="n">
+        <v>9.667</v>
+      </c>
+      <c r="AK13" s="2" t="n">
+        <v>7.639</v>
+      </c>
+      <c r="AL13" s="2" t="n">
+        <v>0.9638</v>
+      </c>
+      <c r="AM13" s="2" t="n">
+        <v>0.3403</v>
+      </c>
+      <c r="AN13" s="2" t="n">
+        <v>0.6228</v>
+      </c>
+      <c r="AO13" s="2" t="n">
+        <v>28.649</v>
+      </c>
+      <c r="AP13" s="2" t="n">
+        <v>29.088</v>
+      </c>
+      <c r="AQ13" s="2" t="n">
+        <v>44.939</v>
+      </c>
+      <c r="AR13" s="2" t="n">
+        <v>15.851</v>
+      </c>
+      <c r="AS13" s="2" t="n">
+        <v>23.416</v>
+      </c>
+      <c r="AT13" s="2" t="n">
+        <v>346.06</v>
+      </c>
+      <c r="AU13" s="2" t="n">
+        <v>118.1</v>
+      </c>
+      <c r="AV13" s="2" t="n">
+        <v>165.154</v>
+      </c>
+      <c r="AW13" s="2" t="n">
+        <v>246.309</v>
+      </c>
+      <c r="AX13" s="2" t="n">
+        <v>262.792</v>
+      </c>
+      <c r="AY13" s="2" t="n">
+        <v>167.181</v>
+      </c>
+      <c r="AZ13" s="2" t="n">
+        <v>700.5</v>
+      </c>
+      <c r="BA13" s="2" t="n">
+        <v>654.4</v>
+      </c>
+      <c r="BB13" s="2" t="n">
+        <v>0.526</v>
+      </c>
+      <c r="BC13" s="2" t="n">
+        <v>0.4895</v>
+      </c>
+      <c r="BD13" s="2" t="n">
+        <v>0.5182</v>
+      </c>
+      <c r="BE13" s="2" t="n">
+        <v>0.4798</v>
+      </c>
+      <c r="BF13" s="2" t="n">
+        <v>0.5108</v>
+      </c>
+      <c r="BG13" s="2" t="n">
+        <v>0.4717</v>
+      </c>
+      <c r="BH13" s="2" t="n">
+        <v>0.9277</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0.7663</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>0.7401</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>0.713</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>345.06</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>124.2</v>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>0.8213</v>
       </c>
-      <c r="I12" s="2" t="n">
-        <v>0.2865</v>
-      </c>
-      <c r="J12" s="2" t="n">
+      <c r="I14" s="2" t="n">
+        <v>0.2957</v>
+      </c>
+      <c r="J14" s="2" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K14" s="2" t="n">
         <v>0.55</v>
       </c>
-      <c r="L12" s="2" t="n">
-        <v>0.9427</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>51.159</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>42297.467</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>39759.619</v>
-      </c>
-      <c r="P12" s="2" t="n">
-        <v>32653.126</v>
-      </c>
-      <c r="Q12" s="2" t="n">
-        <v>735.8</v>
-      </c>
-      <c r="R12" s="2" t="n">
-        <v>1564.88</v>
-      </c>
-      <c r="S12" s="2" t="n">
-        <v>1834.831</v>
-      </c>
-      <c r="T12" s="2" t="n">
-        <v>1.1725</v>
-      </c>
-      <c r="U12" s="2" t="n">
-        <v>481.419</v>
-      </c>
-      <c r="V12" s="2" t="n">
-        <v>7.38</v>
-      </c>
-      <c r="W12" s="2" t="n">
-        <v>0.9718</v>
-      </c>
-      <c r="X12" s="2" t="n">
-        <v>0.2899</v>
-      </c>
-      <c r="Y12" s="2" t="n">
-        <v>0.3563</v>
-      </c>
-      <c r="Z12" s="2" t="n">
-        <v>0.0594</v>
-      </c>
-      <c r="AA12" s="2" t="n">
-        <v>0.2503</v>
-      </c>
-      <c r="AB12" s="2" t="n">
-        <v>0.0562</v>
-      </c>
-      <c r="AC12" s="2" t="n">
-        <v>0.9455</v>
-      </c>
-      <c r="AD12" s="2" t="n">
-        <v>0.9731</v>
-      </c>
-      <c r="AE12" s="2" t="n">
-        <v>369.96</v>
-      </c>
-      <c r="AF12" s="2" t="n">
-        <v>0.2899</v>
-      </c>
-      <c r="AG12" s="2" t="n">
+      <c r="L14" s="2" t="n">
+        <v>0.9304</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>51.971</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>36140.598</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>33972.162</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>27900.099</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>732.1</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>1602.645</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>1836.26</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>1.1458</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>481.98</v>
+      </c>
+      <c r="V14" s="2" t="n">
+        <v>7.605</v>
+      </c>
+      <c r="W14" s="2" t="n">
+        <v>0.9658</v>
+      </c>
+      <c r="X14" s="2" t="n">
+        <v>0.2816</v>
+      </c>
+      <c r="Y14" s="2" t="n">
+        <v>0.3272</v>
+      </c>
+      <c r="Z14" s="2" t="n">
+        <v>0.0619</v>
+      </c>
+      <c r="AA14" s="2" t="n">
+        <v>0.2319</v>
+      </c>
+      <c r="AB14" s="2" t="n">
+        <v>0.0602</v>
+      </c>
+      <c r="AC14" s="2" t="n">
+        <v>0.9321</v>
+      </c>
+      <c r="AD14" s="2" t="n">
+        <v>0.9667</v>
+      </c>
+      <c r="AE14" s="2" t="n">
+        <v>344.42</v>
+      </c>
+      <c r="AF14" s="2" t="n">
+        <v>0.2816</v>
+      </c>
+      <c r="AG14" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="AH12" s="2" t="n">
-        <v>0.3331</v>
-      </c>
-      <c r="AI12" s="2" t="n">
-        <v>123.6</v>
-      </c>
-      <c r="AJ12" s="2" t="n">
+      <c r="AH14" s="2" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="AI14" s="2" t="n">
+        <v>114.2</v>
+      </c>
+      <c r="AJ14" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="AK12" s="2" t="n">
-        <v>8.448</v>
-      </c>
-      <c r="AL12" s="2" t="n">
-        <v>0.9724</v>
-      </c>
-      <c r="AM12" s="2" t="n">
-        <v>0.3331</v>
-      </c>
-      <c r="AN12" s="2" t="n">
-        <v>0.5843</v>
-      </c>
-      <c r="AO12" s="2" t="n">
-        <v>29.683</v>
-      </c>
-      <c r="AP12" s="2" t="n">
-        <v>27.832</v>
-      </c>
-      <c r="AQ12" s="2" t="n">
-        <v>40.632</v>
-      </c>
-      <c r="AR12" s="2" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="AS12" s="2" t="n">
-        <v>60.317</v>
-      </c>
-      <c r="AT12" s="2" t="n">
-        <v>370.51</v>
-      </c>
-      <c r="AU12" s="2" t="n">
-        <v>123.6</v>
-      </c>
-      <c r="AV12" s="2" t="n">
-        <v>171.507</v>
-      </c>
-      <c r="AW12" s="2" t="n">
-        <v>249.563</v>
-      </c>
-      <c r="AX12" s="2" t="n">
-        <v>286.125</v>
-      </c>
-      <c r="AY12" s="2" t="n">
-        <v>189.782</v>
-      </c>
-      <c r="AZ12" s="2" t="n">
-        <v>735.8</v>
-      </c>
-      <c r="BA12" s="2" t="n">
-        <v>685.2</v>
-      </c>
-      <c r="BB12" s="2" t="n">
-        <v>0.5618</v>
-      </c>
-      <c r="BC12" s="2" t="n">
-        <v>0.4881</v>
-      </c>
-      <c r="BD12" s="2" t="n">
-        <v>0.5521</v>
-      </c>
-      <c r="BE12" s="2" t="n">
-        <v>0.4748</v>
-      </c>
-      <c r="BF12" s="2" t="n">
-        <v>0.5545</v>
-      </c>
-      <c r="BG12" s="2" t="n">
-        <v>0.4747</v>
-      </c>
-      <c r="BH12" s="2" t="n">
-        <v>0.9441000000000001</v>
+      <c r="AK14" s="2" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="AL14" s="2" t="n">
+        <v>0.9663</v>
+      </c>
+      <c r="AM14" s="2" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="AN14" s="2" t="n">
+        <v>0.5874</v>
+      </c>
+      <c r="AO14" s="2" t="n">
+        <v>29.401</v>
+      </c>
+      <c r="AP14" s="2" t="n">
+        <v>27.749</v>
+      </c>
+      <c r="AQ14" s="2" t="n">
+        <v>41.149</v>
+      </c>
+      <c r="AR14" s="2" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="AS14" s="2" t="n">
+        <v>60.599</v>
+      </c>
+      <c r="AT14" s="2" t="n">
+        <v>344.74</v>
+      </c>
+      <c r="AU14" s="2" t="n">
+        <v>114.2</v>
+      </c>
+      <c r="AV14" s="2" t="n">
+        <v>157.701</v>
+      </c>
+      <c r="AW14" s="2" t="n">
+        <v>232.67</v>
+      </c>
+      <c r="AX14" s="2" t="n">
+        <v>266.8</v>
+      </c>
+      <c r="AY14" s="2" t="n">
+        <v>173.584</v>
+      </c>
+      <c r="AZ14" s="2" t="n">
+        <v>732.1</v>
+      </c>
+      <c r="BA14" s="2" t="n">
+        <v>689</v>
+      </c>
+      <c r="BB14" s="2" t="n">
+        <v>0.5195</v>
+      </c>
+      <c r="BC14" s="2" t="n">
+        <v>0.4525</v>
+      </c>
+      <c r="BD14" s="2" t="n">
+        <v>0.5134</v>
+      </c>
+      <c r="BE14" s="2" t="n">
+        <v>0.4425</v>
+      </c>
+      <c r="BF14" s="2" t="n">
+        <v>0.5115</v>
+      </c>
+      <c r="BG14" s="2" t="n">
+        <v>0.4372</v>
+      </c>
+      <c r="BH14" s="2" t="n">
+        <v>0.9313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated export of files
</commit_message>
<xml_diff>
--- a/export/Приложение_А.xlsx
+++ b/export/Приложение_А.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Приложение А" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Приложение А" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>